<commit_message>
Consolida busca de sensibilidade IA/ML no núcleo temático (104 → 121)
Integra a RQ6, amplia o núcleo temático para 121 registros, documenta integralmente as strings da Scopus, Web of Science All Databases e Crossref, e atualiza artigo, pipeline, verificadores, PDF, Word e produtos de auditoria.
</commit_message>
<xml_diff>
--- a/referencias/lista_referencias.xlsx
+++ b/referencias/lista_referencias.xlsx
@@ -417,10 +417,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -644,7 +644,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>aliu_barreirasdt_2025</t>
+          <t>alici_iotambientes_2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -654,54 +654,50 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Aliu, Abdulmalik Adozuka and Ariff, Nor Rima Muhamad and Said, Sheikh Ali Azzran Sh and Ametefe, Divine Senanu and John, Dah</t>
+          <t>Alici, Nedim</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Barriers to digital transformation in facilities management: insights from a developing country</t>
+          <t>IoT-enabled indoor environments in smart cities: a systematic review on energy efficiency, user comfort, and environmental sustainability</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Journal of Construction in Developing Countries</t>
+          <t>Frontiers in Sustainability</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>137-168</t>
+          <t>1751337</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>10.21315/jcdc.2025.30.2.6</t>
+          <t>10.3389/frsus.2026.1751337</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.21315/jcdc.2025.30.2.6</t>
+          <t>https://doi.org/10.3389/frsus.2026.1751337</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>araujoneto_manutencaolegislacao_2015</t>
+          <t>aliu_barreirasdt_2025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -711,54 +707,54 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Araújo Neto, Paschoal Gavazza de</t>
+          <t>Aliu, Abdulmalik Adozuka and Ariff, Nor Rima Muhamad and Said, Sheikh Ali Azzran Sh and Ametefe, Divine Senanu and John, Dah</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>A manutenção predial nas edificações públicas, um estudo sobre a legislação</t>
+          <t>Barriers to digital transformation in facilities management: insights from a developing country</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>E\&amp;S Engineering and Science</t>
+          <t>Journal of Construction in Developing Countries</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>85-93</t>
+          <t>137-168</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>10.18607/ES201532557</t>
+          <t>10.21315/jcdc.2025.30.2.6</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://doi.org/10.18607/ES201532557</t>
+          <t>https://doi.org/10.21315/jcdc.2025.30.2.6</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>awuzie_fmuniversidades_2017</t>
+          <t>araujoneto_manutencaolegislacao_2015</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -768,54 +764,54 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Awuzie, Bankole Osita and Isa, Rasheed</t>
+          <t>Araújo Neto, Paschoal Gavazza de</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Stakeholders' perception of critical success factors for sustainable facilities management practice in universities in sub-Saharan Africa</t>
+          <t>A manutenção predial nas edificações públicas, um estudo sobre a legislação</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Acta Structilia</t>
+          <t>E\&amp;S Engineering and Science</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>106-127</t>
+          <t>85-93</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>10.18820/24150487/as24i2.4</t>
+          <t>10.18607/ES201532557</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://doi.org/10.18820/24150487/as24i2.4</t>
+          <t>https://doi.org/10.18607/ES201532557</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>chew_manutenibilidadeverde_2016</t>
+          <t>awuzie_fmuniversidades_2017</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -825,54 +821,54 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chew, Michael Yit Lin and Conejos, Sheila</t>
+          <t>Awuzie, Bankole Osita and Isa, Rasheed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Developing a green maintainability framework for green walls in Singapore</t>
+          <t>Stakeholders' perception of critical success factors for sustainable facilities management practice in universities in sub-Saharan Africa</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Structural Survey</t>
+          <t>Acta Structilia</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>24</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>379-406</t>
+          <t>106-127</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>10.1108/SS-02-2016-0007</t>
+          <t>10.18820/24150487/as24i2.4</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/SS-02-2016-0007</t>
+          <t>https://doi.org/10.18820/24150487/as24i2.4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>conejos_verticalgreenery_2019</t>
+          <t>barbosa_facilitiesinstituicaopublica_2020</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -882,87 +878,111 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Conejos, Sheila and Chew, Michael Yit Lin and Azril, Fikril Hakim Bin</t>
+          <t>Barbosa, Ana Maria da Silva and Jerônimo, Taciana de Barros and Ramos, Patrícia Tatiana Ferreira and Santos, Juliana Karla Rodrigues de Souza</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Green maintainability assessment of high-rise vertical greenery systems</t>
+          <t>A gestão de facilities na manutenção de uma instituição pública</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Revista Gestão Industrial</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1008-1047</t>
+          <t>129-146</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>10.1108/F-09-2018-0107</t>
+          <t>10.3895/gi.v16n3.8968</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/F-09-2018-0107</t>
+          <t>https://doi.org/10.3895/gi.v16n3.8968</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>crossref_restapi_2026</t>
+          <t>chew_manutenibilidadeverde_2016</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>article</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{Crossref}</t>
+          <t>Chew, Michael Yit Lin and Conejos, Sheila</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>REST API: metadata retrieval</t>
+          <t>Developing a green maintainability framework for green walls in Singapore</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Structural Survey</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>379-406</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>10.1108/SS-02-2016-0007</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/SS-02-2016-0007</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>deng_bimdigitaltwins_2021</t>
+          <t>conejos_verticalgreenery_2019</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -972,103 +992,87 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Deng, Min and Menassa, Carol C. and Kamat, Vineet R.</t>
+          <t>Conejos, Sheila and Chew, Michael Yit Lin and Azril, Fikril Hakim Bin</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>From BIM to digital twins: a systematic review of the evolution of intelligent building representations in the AEC-FM industry</t>
+          <t>Green maintainability assessment of high-rise vertical greenery systems</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Journal of Information Technology in Construction (ITcon)</t>
+          <t>Facilities</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>58-83</t>
+          <t>1008-1047</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>10.36680/j.itcon.2021.005</t>
+          <t>10.1108/F-09-2018-0107</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://doi.org/10.36680/j.itcon.2021.005</t>
+          <t>https://doi.org/10.1108/F-09-2018-0107</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>donthu_bibliometria_2021</t>
+          <t>crossref_restapi_2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>article</t>
+          <t>online</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Donthu, Naveen and Kumar, Satish and Mukherjee, Debmalya and Pandey, Nitesh and Lim, Weng Marc</t>
+          <t>{Crossref}</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>How to conduct a bibliometric analysis: an overview and guidelines</t>
+          <t>REST API: metadata retrieval</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Journal of Business Research</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>133</t>
-        </is>
-      </c>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>285-296</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>10.1016/j.jbusres.2021.04.070</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.jbusres.2021.04.070</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ferreira_manutencaoceramica_2020</t>
+          <t>das_iotai_2025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1078,54 +1082,54 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ferreira, Cláudia and Neves, Luís Canhoto and Silva, Ana and de Brito, Jorge</t>
+          <t>Das, Dillip Kumar</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Stochastic maintenance models for ceramic claddings</t>
+          <t>Integrating IoT and AI for Sustainable Energy-Efficient Smart Building: Potential, Barriers and Strategic Pathways</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Structure and Infrastructure Engineering</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>247-265</t>
+          <t>10313</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>10.1080/15732479.2019.1652657</t>
+          <t>10.3390/su172210313</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1080/15732479.2019.1652657</t>
+          <t>https://doi.org/10.3390/su172210313</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gispert_ontologiaativos_2025</t>
+          <t>deng_bimdigitaltwins_2021</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1135,54 +1139,50 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Espinosa Gispert, Diego and Yitmen, Ibrahim and Sadri, Habib and Taheri, Afshin</t>
+          <t>Deng, Min and Menassa, Carol C. and Kamat, Vineet R.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Development of an ontology-based asset information model for predictive maintenance in building facilities</t>
+          <t>From BIM to digital twins: a systematic review of the evolution of intelligent building representations in the AEC-FM industry</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Smart and Sustainable Built Environment</t>
+          <t>Journal of Information Technology in Construction (ITcon)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>740-757</t>
+          <t>58-83</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>10.1108/SASBE-07-2023-0170</t>
+          <t>10.36680/j.itcon.2021.005</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/SASBE-07-2023-0170</t>
+          <t>https://doi.org/10.36680/j.itcon.2021.005</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>goretti_bimoem_2023</t>
+          <t>donthu_bibliometria_2021</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1192,50 +1192,50 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Goretti, Hannah A. and Kaming, Peter</t>
+          <t>Donthu, Naveen and Kumar, Satish and Mukherjee, Debmalya and Pandey, Nitesh and Lim, Weng Marc</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A review and bibliometric analysis of utilizing building information modeling (BIM) on effective operation and maintenance (O\&amp;M)</t>
+          <t>How to conduct a bibliometric analysis: an overview and guidelines</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>E3S Web of Conferences</t>
+          <t>Journal of Business Research</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>429</t>
+          <t>133</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>01002</t>
+          <t>285-296</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>10.1051/e3sconf/202342901002</t>
+          <t>10.1016/j.jbusres.2021.04.070</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1051/e3sconf/202342901002</t>
+          <t>https://doi.org/10.1016/j.jbusres.2021.04.070</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hu_revisao_sintese_2026</t>
+          <t>ferreira_manutencaoceramica_2020</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1245,54 +1245,54 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hu, Meilan and Koh, Paye Shin and Soh, Xun Ci and Hartanto, Andree and Majeed, Nadyanna M.</t>
+          <t>Ferreira, Cláudia and Neves, Luís Canhoto and Silva, Ana and de Brito, Jorge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>From review to synthesis: a step-by-step methodological guide to systematic reviews and multilevel meta-analyses</t>
+          <t>Stochastic maintenance models for ceramic claddings</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Behavior Research Methods</t>
+          <t>Structure and Infrastructure Engineering</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>197</t>
+          <t>247-265</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>10.3758/s13428-026-02961-x</t>
+          <t>10.1080/15732479.2019.1652657</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3758/s13428-026-02961-x</t>
+          <t>https://doi.org/10.1080/15732479.2019.1652657</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>jiang_deduplicacao_regras_2014</t>
+          <t>gispert_ontologiaativos_2025</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1302,50 +1302,54 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Jiang, Yu and Lin, Can and Meng, Weiyi and Yu, Clement and Cohen, Aaron M. and Smalheiser, Neil R.</t>
+          <t>Espinosa Gispert, Diego and Yitmen, Ibrahim and Sadri, Habib and Taheri, Afshin</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Rule-based deduplication of article records from bibliographic databases</t>
+          <t>Development of an ontology-based asset information model for predictive maintenance in building facilities</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Smart and Sustainable Built Environment</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2014</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>bat086</t>
+          <t>740-757</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>10.1093/database/bat086</t>
+          <t>10.1108/SASBE-07-2023-0170</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1093/database/bat086</t>
+          <t>https://doi.org/10.1108/SASBE-07-2023-0170</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>kim_estimativacustoseducacional_2018</t>
+          <t>goretti_bimoem_2023</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1355,54 +1359,50 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Kim, Ji-Myong and Kim, Taehui and Yu, Yeong-Jin and Son, Kiyoung</t>
+          <t>Goretti, Hannah A. and Kaming, Peter</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Development of a maintenance and repair cost estimation model for educational buildings using regression analysis</t>
+          <t>A review and bibliometric analysis of utilizing building information modeling (BIM) on effective operation and maintenance (O\&amp;M)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Journal of Asian Architecture and Building Engineering</t>
+          <t>E3S Web of Conferences</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>429</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>307-312</t>
+          <t>01002</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>10.3130/jaabe.17.307</t>
+          <t>10.1051/e3sconf/202342901002</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3130/jaabe.17.307</t>
+          <t>https://doi.org/10.1051/e3sconf/202342901002</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>martins_custosmanutencaoses_2024</t>
+          <t>hu_revisao_sintese_2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1412,54 +1412,54 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Martins, Rafael Fernando Batista and Espejo, Márcia Maria dos Santos Bortolocci</t>
+          <t>Hu, Meilan and Koh, Paye Shin and Soh, Xun Ci and Hartanto, Andree and Majeed, Nadyanna M.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Análise de custos de manutenção predial em uma universidade federal brasileira com uso do modelo de suavização exponencial simples</t>
+          <t>From review to synthesis: a step-by-step methodological guide to systematic reviews and multilevel meta-analyses</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ABCustos</t>
+          <t>Behavior Research Methods</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>58</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>79-98</t>
+          <t>197</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>10.47179/abcustos.v19i1.719</t>
+          <t>10.3758/s13428-026-02961-x</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://doi.org/10.47179/abcustos.v19i1.719</t>
+          <t>https://doi.org/10.3758/s13428-026-02961-x</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>masmoudi_ahptopsis_2026</t>
+          <t>jiang_deduplicacao_regras_2014</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1469,54 +1469,50 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Masmoudi, Malek and Alshamsi, Mohamed and Piya, Sujan and Gupta, Srikant</t>
+          <t>Jiang, Yu and Lin, Can and Meng, Weiyi and Yu, Clement and Cohen, Aaron M. and Smalheiser, Neil R.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Contractors allocation for public building maintenance: a sustainable approach aligned with SDGs using AHP-TOPSIS and bi-objective optimization</t>
+          <t>Rule-based deduplication of article records from bibliographic databases</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2014</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>International Transactions in Operational Research</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2535-2576</t>
+          <t>bat086</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10.1111/itor.70022</t>
+          <t>10.1093/database/bat086</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/itor.70022</t>
+          <t>https://doi.org/10.1093/database/bat086</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>morais_eficienciamanutencao_2023</t>
+          <t>kim_estimativacustoseducacional_2018</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1526,54 +1522,54 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Morais, Lucas Salomão Rael de and Paula, Heber Martins de and Reis, Ricardo Prado Abreu</t>
+          <t>Kim, Ji-Myong and Kim, Taehui and Yu, Yeong-Jin and Son, Kiyoung</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Promoção da eficiência da manutenção predial em edificações públicas: abordagem baseada em registros de ordens de serviço</t>
+          <t>Development of a maintenance and repair cost estimation model for educational buildings using regression analysis</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Paranoá</t>
+          <t>Journal of Asian Architecture and Building Engineering</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1-27</t>
+          <t>307-312</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>10.18830/issn.1679-0944.n34.2023.08</t>
+          <t>10.3130/jaabe.17.307</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://doi.org/10.18830/issn.1679-0944.n34.2023.08</t>
+          <t>https://doi.org/10.3130/jaabe.17.307</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>nageli_ciclovida_2019</t>
+          <t>lateef_manutencaouniversidade_2010</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1583,50 +1579,46 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nägeli, Claudio and Farahani, Abolfazl and Österbring, Magnus and Dalenbäck, Jan-Olof and Wallbaum, Holger</t>
+          <t>Lateef, Olanrewaju Abdul and Khamidi, Mohd Faris and Idrus, Arazi</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A service-life cycle approach to maintenance and energy retrofit planning for building portfolios</t>
+          <t>Building maintenance management in a Malaysian university campuses: a case study</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Building and Environment</t>
+          <t>Australasian Journal of Construction Economics and Building</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>106212</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>10.1016/j.buildenv.2019.106212</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.buildenv.2019.106212</t>
-        </is>
-      </c>
+          <t>76-89</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>naji_campusdelphi_2023</t>
+          <t>maia_gestaoinformacaomanutencao_2016</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1636,54 +1628,46 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Naji, Khalid K. and Gunduz, Murat and Maki, Omar</t>
+          <t>Maia, Barbara Lepca and Scheer, Sérgio and Freitas, Maria do Carmo Duarte</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Development of a campus facility management operational framework using a modified Delphi method</t>
+          <t>Manutenção predial: a prospecta de decisões a partir da gestão da informação</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Journal of Construction Engineering and Management</t>
+          <t>Revista de Engenharia e Tecnologia</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>04023052</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>10.1061/JCEMD4.COENG-13154</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1061/JCEMD4.COENG-13154</t>
-        </is>
-      </c>
+          <t>37-55</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ndukuba_resilienciainstitucional_2025</t>
+          <t>martins_custosmanutencaoses_2024</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1693,54 +1677,54 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ndukuba, Samuel Nnadoziem</t>
+          <t>Martins, Rafael Fernando Batista and Espejo, Márcia Maria dos Santos Bortolocci</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Building institutional resilience through sustainable facility management in South African vocational education</t>
+          <t>Análise de custos de manutenção predial em uma universidade federal brasileira com uso do modelo de suavização exponencial simples</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Construction Entrepreneurship and Real Property</t>
+          <t>ABCustos</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>110-123</t>
+          <t>79-98</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>10.56065/pdpyke84</t>
+          <t>10.47179/abcustos.v19i1.719</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://doi.org/10.56065/pdpyke84</t>
+          <t>https://doi.org/10.47179/abcustos.v19i1.719</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>nielsen_sustentabilidadefm_2016</t>
+          <t>masmoudi_ahptopsis_2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1750,54 +1734,54 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Nielsen, Susanne Balslev and Sarasoja, Anna-Liisa and Galamba, Kirsten Ramskov</t>
+          <t>Masmoudi, Malek and Alshamsi, Mohamed and Piya, Sujan and Gupta, Srikant</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sustainability in facilities management: an overview of current research</t>
+          <t>Contractors allocation for public building maintenance: a sustainable approach aligned with SDGs using AHP-TOPSIS and bi-objective optimization</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>International Transactions in Operational Research</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>33</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>9-10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>535-563</t>
+          <t>2535-2576</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>10.1108/F-07-2014-0060</t>
+          <t>10.1111/itor.70022</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/F-07-2014-0060</t>
+          <t>https://doi.org/10.1111/itor.70022</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>okoro_sustainablefm_2023</t>
+          <t>morais_eficienciamanutencao_2023</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1807,12 +1791,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Okoro, Chioma Sylvia</t>
+          <t>Morais, Lucas Salomão Rael de and Paula, Heber Martins de and Reis, Ricardo Prado Abreu</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sustainable facilities management in the built environment: a mixed-method review</t>
+          <t>Promoção da eficiência da manutenção predial em edificações públicas: abordagem baseada em registros de ordens de serviço</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1822,39 +1806,39 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Paranoá</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>3174</t>
+          <t>1-27</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>10.3390/su15043174</t>
+          <t>10.18830/issn.1679-0944.n34.2023.08</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/su15043174</t>
+          <t>https://doi.org/10.18830/issn.1679-0944.n34.2023.08</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>opoku_futurofm_2022</t>
+          <t>motuziene_ventilacaoia_2025</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1864,17 +1848,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Opoku, Alex and Lee, Jeoung Yul</t>
+          <t>Motuzienė, Violeta and Bielskus, Jonas and Džiugaitė-Tumėnienė, Rasa and Raudonis, Vidas</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>The future of facilities management: managing facilities for sustainable development</t>
+          <t>Occupancy-Based Predictive AI-Driven Ventilation Control for Energy Savings in Office Buildings</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1884,34 +1868,34 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1705</t>
+          <t>4140</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>10.3390/su14031705</t>
+          <t>10.3390/su17094140</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/su14031705</t>
+          <t>https://doi.org/10.3390/su17094140</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>othman_manutenibilidadeesi_2023</t>
+          <t>nageli_ciclovida_2019</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1921,50 +1905,50 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Othman, Ayman Ahmed Ezzat and Kamal, Ahmed</t>
+          <t>Nägeli, Claudio and Farahani, Abolfazl and Österbring, Magnus and Dalenbäck, Jan-Olof and Wallbaum, Holger</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Enhancing building maintainability through early supplier involvement in the design process</t>
+          <t>A service-life cycle approach to maintenance and energy retrofit planning for building portfolios</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Organization, Technology and Management in Construction</t>
+          <t>Building and Environment</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>160</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>34-49</t>
+          <t>106212</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>10.2478/otmcj-2023-0005</t>
+          <t>10.1016/j.buildenv.2019.106212</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://doi.org/10.2478/otmcj-2023-0005</t>
+          <t>https://doi.org/10.1016/j.buildenv.2019.106212</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>park_cbrfuzzyahp_2019</t>
+          <t>naji_campusdelphi_2023</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1974,54 +1958,54 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Park, Sojin and Kwon, Nahyun and Ahn, Yonghan</t>
+          <t>Naji, Khalid K. and Gunduz, Murat and Maki, Omar</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Forecasting Repair Schedule for Building Components Based on Case-Based Reasoning and Fuzzy-AHP</t>
+          <t>Development of a campus facility management operational framework using a modified Delphi method</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sustainability</t>
+          <t>Journal of Construction Engineering and Management</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>149</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>7181</t>
+          <t>04023052</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>10.3390/su11247181</t>
+          <t>10.1061/JCEMD4.COENG-13154</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/su11247181</t>
+          <t>https://doi.org/10.1061/JCEMD4.COENG-13154</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ramantswana_esgfm_2026</t>
+          <t>ndukuba_resilienciainstitucional_2025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2031,54 +2015,54 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ramantswana, Thabelo and Awuzie, Bankole and Mompati, Lerato and Khafiso, Thabo</t>
+          <t>Ndukuba, Samuel Nnadoziem</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Embedding ESG in facility management practices: a South African corporate real estate perspective</t>
+          <t>Building institutional resilience through sustainable facility management in South African vocational education</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>International Journal of Building Pathology and Adaptation</t>
+          <t>Construction Entrepreneurship and Real Property</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>1246-1266</t>
+          <t>110-123</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>10.1108/IJBPA-07-2025-0169</t>
+          <t>10.56065/pdpyke84</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/IJBPA-07-2025-0169</t>
+          <t>https://doi.org/10.56065/pdpyke84</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>rathbone_deduplicacao_2015</t>
+          <t>nielsen_sustentabilidadefm_2016</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2088,50 +2072,54 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Rathbone, John and Carter, Matt and Hoffmann, Tammy and Glasziou, Paul</t>
+          <t>Nielsen, Susanne Balslev and Sarasoja, Anna-Liisa and Galamba, Kirsten Ramskov</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Better duplicate detection for systematic reviewers: evaluation of Systematic Review Assistant-Deduplication Module</t>
+          <t>Sustainability in facilities management: an overview of current research</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Systematic Reviews</t>
+          <t>Facilities</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>9-10</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>535-563</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>10.1186/2046-4053-4-6</t>
+          <t>10.1108/F-07-2014-0060</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1186/2046-4053-4-6</t>
+          <t>https://doi.org/10.1108/F-07-2014-0060</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>snyder_revisaometodologia_2019</t>
+          <t>okoro_sustainablefm_2023</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2141,50 +2129,54 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Snyder, Hannah</t>
+          <t>Okoro, Chioma Sylvia</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Literature review as a research methodology: an overview and guidelines</t>
+          <t>Sustainable facilities management in the built environment: a mixed-method review</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Journal of Business Research</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>104</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>333-339</t>
+          <t>3174</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>10.1016/j.jbusres.2019.07.039</t>
+          <t>10.3390/su15043174</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jbusres.2019.07.039</t>
+          <t>https://doi.org/10.3390/su15043174</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>talib_hospitalfm_2013</t>
+          <t>opoku_futurofm_2022</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2194,54 +2186,54 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Talib, Yuhainis and Rajagopalan, Priyadarsini and Yang, Jay</t>
+          <t>Opoku, Alex and Lee, Jeoung Yul</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Evaluation of building performance for strategic facilities management in healthcare: a case study of a public hospital in Australia</t>
+          <t>The future of facilities management: managing facilities for sustainable development</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2013</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>681-701</t>
+          <t>1705</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>10.1108/F-06-2012-0042</t>
+          <t>10.3390/su14031705</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/F-06-2012-0042</t>
+          <t>https://doi.org/10.3390/su14031705</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>tan_fluxoinformacao_2018</t>
+          <t>othman_manutenibilidadeesi_2023</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2251,54 +2243,50 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tan, Adeline Zhu Teng and Zaman, Atiq Uz and Sutrisna, Monty</t>
+          <t>Othman, Ayman Ahmed Ezzat and Kamal, Ahmed</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Enabling an effective knowledge and information flow between the phases of building construction and facilities management</t>
+          <t>Enhancing building maintainability through early supplier involvement in the design process</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Facilities</t>
+          <t>Organization, Technology and Management in Construction</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>3/4</t>
-        </is>
-      </c>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>151-170</t>
+          <t>34-49</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>10.1108/F-03-2016-0028</t>
+          <t>10.2478/otmcj-2023-0005</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1108/F-03-2016-0028</t>
+          <t>https://doi.org/10.2478/otmcj-2023-0005</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>whittemore_revisaointegrativa_2005</t>
+          <t>park_cbrfuzzyahp_2019</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2308,102 +2296,546 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Whittemore, Robin and Knafl, Kathleen</t>
+          <t>Park, Sojin and Kwon, Nahyun and Ahn, Yonghan</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>The integrative review: updated methodology</t>
+          <t>Forecasting Repair Schedule for Building Components Based on Case-Based Reasoning and Fuzzy-AHP</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Journal of Advanced Nursing</t>
+          <t>Sustainability</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>546-553</t>
+          <t>7181</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>10.1111/j.1365-2648.2005.03621.x</t>
+          <t>10.3390/su11247181</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/j.1365-2648.2005.03621.x</t>
+          <t>https://doi.org/10.3390/su11247181</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>ramantswana_esgfm_2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Ramantswana, Thabelo and Awuzie, Bankole and Mompati, Lerato and Khafiso, Thabo</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Embedding ESG in facility management practices: a South African corporate real estate perspective</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>International Journal of Building Pathology and Adaptation</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>1246-1266</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>10.1108/IJBPA-07-2025-0169</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/IJBPA-07-2025-0169</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>rathbone_deduplicacao_2015</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Rathbone, John and Carter, Matt and Hoffmann, Tammy and Glasziou, Paul</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Better duplicate detection for systematic reviewers: evaluation of Systematic Review Assistant-Deduplication Module</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>10.1186/2046-4053-4-6</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/2046-4053-4-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>snyder_revisaometodologia_2019</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Snyder, Hannah</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Literature review as a research methodology: an overview and guidelines</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Journal of Business Research</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>333-339</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>10.1016/j.jbusres.2019.07.039</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jbusres.2019.07.039</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>suh_demandaenergiaagua_2012</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Suh, Dongjun and Chang, Seongju</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>An Energy and Water Resource Demand Estimation Model for Multi-Family Housing Complexes in Korea</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Energies</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>4497-4516</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>10.3390/en5114497</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en5114497</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>talib_hospitalfm_2013</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Talib, Yuhainis and Rajagopalan, Priyadarsini and Yang, Jay</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Evaluation of building performance for strategic facilities management in healthcare: a case study of a public hospital in Australia</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>13/14</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>681-701</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>10.1108/F-06-2012-0042</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/F-06-2012-0042</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>tan_fluxoinformacao_2018</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tan, Adeline Zhu Teng and Zaman, Atiq Uz and Sutrisna, Monty</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Enabling an effective knowledge and information flow between the phases of building construction and facilities management</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>151-170</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>10.1108/F-03-2016-0028</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/F-03-2016-0028</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>whittemore_revisaointegrativa_2005</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Whittemore, Robin and Knafl, Kathleen</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>The integrative review: updated methodology</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Journal of Advanced Nursing</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>546-553</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>10.1111/j.1365-2648.2005.03621.x</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/j.1365-2648.2005.03621.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>wu_gnnvidautil_2025</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Wu, Pei-Yu and Mundt-Petersen, S. Olof</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Empirical Quantification and Prediction of Building Component Lifespans with Graph Neural Networks</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>IOP Conference Series: Earth and Environmental Science</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>1554</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>012036</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>10.1088/1755-1315/1554/1/012036</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1088/1755-1315/1554/1/012036</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>yoon_fuzzyfm_2018</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
         <is>
           <t>Yoon, Jong Han and Cha, Hee Sung</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Optimal FM Strategy for Commercial Office Buildings Using Fuzzy Synthetic Evaluation</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Journal of Performance of Constructed Facilities</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>04018025</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>10.1061/(ASCE)CF.1943-5509.0001176</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>https://doi.org/10.1061/(ASCE)CF.1943-5509.0001176</t>
         </is>

</xml_diff>